<commit_message>
Derniere fiinalisation todo xlsx
</commit_message>
<xml_diff>
--- a/ToDo.xlsx
+++ b/ToDo.xlsx
@@ -1,46 +1,36 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr hidePivotFieldList="1"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Cours\Web_Avance_Mr_Rojo\Examen\Iran\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C602C5-A6AC-47AE-AA47-AB353195EB52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
-  <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
-  </bookViews>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <workbookPr/>
   <sheets>
-    <sheet name="groupe" sheetId="1" r:id="rId1"/>
-    <sheet name="liste des taches" sheetId="2" r:id="rId2"/>
-    <sheet name="Recap" sheetId="3" r:id="rId3"/>
-    <sheet name="avancement" sheetId="4" r:id="rId4"/>
-    <sheet name="detail_avancement" sheetId="5" r:id="rId5"/>
+    <sheet state="visible" name="groupe" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="liste des taches" sheetId="2" r:id="rId6"/>
+    <sheet state="visible" name="Recap" sheetId="3" r:id="rId7"/>
+    <sheet state="visible" name="avancement" sheetId="4" r:id="rId8"/>
+    <sheet state="visible" name="detail_avancement" sheetId="5" r:id="rId9"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <definedNames/>
+  <calcPr/>
   <pivotCaches>
-    <pivotCache cacheId="4" r:id="rId6"/>
+    <pivotCache cacheId="0" r:id="rId10"/>
   </pivotCaches>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="95">
+  <si>
+    <t>ETU003268</t>
+  </si>
+  <si>
+    <t>Harena</t>
+  </si>
+  <si>
+    <t>ETU003310</t>
+  </si>
+  <si>
+    <t>Fifaliana</t>
+  </si>
   <si>
     <t>Ligne</t>
   </si>
@@ -75,61 +65,211 @@
     <t>Avancement</t>
   </si>
   <si>
+    <t>Infrastructure</t>
+  </si>
+  <si>
+    <t>Setup</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Init dépôt Git + structure dossiers PHP</t>
+  </si>
+  <si>
+    <t>Technique</t>
+  </si>
+  <si>
+    <t>Docker</t>
+  </si>
+  <si>
+    <t>Dockerfile (PHP + Apache) + docker-compose</t>
+  </si>
+  <si>
+    <t>Base de données</t>
+  </si>
+  <si>
+    <t>Modélisation</t>
+  </si>
+  <si>
+    <t>Schéma DB : tables articles, catégories, images</t>
+  </si>
+  <si>
+    <t>Base</t>
+  </si>
+  <si>
+    <t>Script SQL de création + données de test</t>
+  </si>
+  <si>
     <t>Backoffice</t>
   </si>
   <si>
-    <t>Gestion article</t>
-  </si>
-  <si>
-    <t>Article-add</t>
-  </si>
-  <si>
-    <t>Ajout article : code html + images + articles references</t>
+    <t>Utilisateurs</t>
+  </si>
+  <si>
+    <t>register.php</t>
+  </si>
+  <si>
+    <t>Formulaire d'inscription + hashage mot de passe</t>
+  </si>
+  <si>
+    <t>Métier</t>
+  </si>
+  <si>
+    <t>login.php</t>
+  </si>
+  <si>
+    <t>Page de connexion + vérification session</t>
+  </si>
+  <si>
+    <t>Sécurité</t>
+  </si>
+  <si>
+    <t>logout.php</t>
+  </si>
+  <si>
+    <t>Destruction de la session</t>
+  </si>
+  <si>
+    <t>Sécurisation de toutes les pages BO (check session)</t>
+  </si>
+  <si>
+    <t>Gestion Catégorie</t>
+  </si>
+  <si>
+    <t>categorie.php</t>
+  </si>
+  <si>
+    <t>Liste des catégories</t>
   </si>
   <si>
     <t>Affichage</t>
   </si>
   <si>
-    <t>Traitement-add</t>
-  </si>
-  <si>
-    <t>Conversion en html avec tinymce</t>
-  </si>
-  <si>
-    <t>Metier</t>
-  </si>
-  <si>
-    <t>Upload images</t>
-  </si>
-  <si>
-    <t>Ajout article : code html en base +articles references en base</t>
-  </si>
-  <si>
-    <t>Appelle de fonctions du DAO</t>
-  </si>
-  <si>
-    <t>Integration</t>
-  </si>
-  <si>
-    <t>Gestion Categorie</t>
-  </si>
-  <si>
-    <t>Categorie</t>
-  </si>
-  <si>
-    <t>Liste</t>
-  </si>
-  <si>
-    <t>Categorie-add</t>
-  </si>
-  <si>
-    <t>Ajout</t>
-  </si>
-  <si>
-    <t>ETU00YYYY</t>
-  </si>
-  <si>
-    <t>Base</t>
+    <t>categorie-add.php</t>
+  </si>
+  <si>
+    <t>Ajout catégorie : formulaire HTML</t>
+  </si>
+  <si>
+    <t>traitement-categorie.php</t>
+  </si>
+  <si>
+    <t>Traitement ajout catégorie en base</t>
+  </si>
+  <si>
+    <t>categorie-edit.php</t>
+  </si>
+  <si>
+    <t>Modification/suppression catégorie</t>
+  </si>
+  <si>
+    <t>Gestion Article</t>
+  </si>
+  <si>
+    <t>article-add.php</t>
+  </si>
+  <si>
+    <t>Formulaire ajout article : champs HTML + images + articles référencés</t>
+  </si>
+  <si>
+    <t>Intégration TinyMCE pour saisie HTML du contenu</t>
+  </si>
+  <si>
+    <t>traitement-add.php</t>
+  </si>
+  <si>
+    <t>Upload images sur serveur</t>
+  </si>
+  <si>
+    <t>Insertion article en base (contenu HTML + images + références)</t>
+  </si>
+  <si>
+    <t>article-list.php</t>
+  </si>
+  <si>
+    <t>Liste articles + boutons édition/suppression</t>
+  </si>
+  <si>
+    <t>article-edit.php</t>
+  </si>
+  <si>
+    <t>Modification article (TinyMCE + images)</t>
+  </si>
+  <si>
+    <t>Frontoffice</t>
+  </si>
+  <si>
+    <t>Structure</t>
+  </si>
+  <si>
+    <t>layout.php</t>
+  </si>
+  <si>
+    <t>Gabarit commun (header, nav, footer) avec h1-h6 sémantiques</t>
+  </si>
+  <si>
+    <t>Accueil</t>
+  </si>
+  <si>
+    <t>index.php</t>
+  </si>
+  <si>
+    <t>Liste articles par catégorie</t>
+  </si>
+  <si>
+    <t>Article</t>
+  </si>
+  <si>
+    <t>article.php</t>
+  </si>
+  <si>
+    <t>Affichage article complet + articles référencés</t>
+  </si>
+  <si>
+    <t>SEO</t>
+  </si>
+  <si>
+    <t>.htaccess</t>
+  </si>
+  <si>
+    <t>URL Rewriting (ex: /article/guerre-iran-2024)</t>
+  </si>
+  <si>
+    <t>toutes pages</t>
+  </si>
+  <si>
+    <t>Balises méta dynamiques (title, description)</t>
+  </si>
+  <si>
+    <t>Alt sur toutes les images</t>
+  </si>
+  <si>
+    <t>Livraison</t>
+  </si>
+  <si>
+    <t>Audit</t>
+  </si>
+  <si>
+    <t>Test Lighthouse mobile + desktop (score ≥ 90)</t>
+  </si>
+  <si>
+    <t>Intégration</t>
+  </si>
+  <si>
+    <t>Documentation</t>
+  </si>
+  <si>
+    <t>doc-technique.pdf</t>
+  </si>
+  <si>
+    <t>Captures FO/BO, schéma DB, identifiants BO, numéros ETU</t>
+  </si>
+  <si>
+    <t>Packaging</t>
+  </si>
+  <si>
+    <t>ZIP du projet fonctionnel + lien dépôt public Git</t>
   </si>
   <si>
     <t>SUM of Estimation</t>
@@ -141,6 +281,9 @@
     <t>SUM of Reste à faire</t>
   </si>
   <si>
+    <t>Total général</t>
+  </si>
+  <si>
     <t>estimation total</t>
   </si>
   <si>
@@ -160,110 +303,108 @@
   </si>
   <si>
     <t>Total</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>(blank)</t>
-  </si>
-  <si>
-    <t>Grand Total</t>
-  </si>
-  <si>
-    <t>ETU003268</t>
-  </si>
-  <si>
-    <t>Harena</t>
-  </si>
-  <si>
-    <t>ETU003310</t>
-  </si>
-  <si>
-    <t>Fifaliana</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="d/m"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="14">
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <color theme="1"/>
+      <name val="Liberation Serif"/>
+    </font>
+    <font>
+      <color rgb="FF000000"/>
+      <name val="&quot;Segoe WPC&quot;"/>
+    </font>
+    <font>
       <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="11"/>
       <color rgb="FF000000"/>
-      <name val="Liberation Serif"/>
+      <name val="&quot;Segoe WPC&quot;"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10.0"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Liberation Serif"/>
-    </font>
-    <font>
       <b/>
-      <sz val="10"/>
+      <sz val="10.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
     </font>
     <font>
       <b/>
-      <sz val="12"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="12"/>
+      <sz val="12.0"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125"/>
+      <patternFill patternType="lightGray"/>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFC9DAF8"/>
-        <bgColor rgb="FFC9DAF8"/>
+        <fgColor rgb="FF252526"/>
+        <bgColor rgb="FF252526"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor rgb="FF000000"/>
       </patternFill>
     </fill>
     <fill>
@@ -279,14 +420,8 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
+  <borders count="15">
+    <border/>
     <border>
       <left style="thin">
         <color rgb="FF000000"/>
@@ -300,40 +435,51 @@
       <bottom style="thin">
         <color rgb="FF000000"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
+      <left style="thin">
+        <color rgb="FF6B7280"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF6B7280"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF6B7280"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF6B7280"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF6B7280"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF6B7280"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF6B7280"/>
+      </top>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF999999"/>
       </left>
-      <right/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="65"/>
+        <color rgb="FFFFFFFF"/>
       </left>
-      <right/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
-        <color indexed="65"/>
+        <color rgb="FFFFFFFF"/>
       </left>
       <right style="thin">
         <color rgb="FF999999"/>
@@ -341,73 +487,50 @@
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF999999"/>
       </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
     </border>
     <border>
       <left style="thin">
         <color rgb="FF999999"/>
       </left>
-      <right/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
-      <right/>
       <top style="thin">
         <color rgb="FF999999"/>
       </top>
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
-      <diagonal/>
     </border>
     <border>
-      <left/>
       <right style="thin">
         <color rgb="FF999999"/>
       </right>
@@ -417,82 +540,227 @@
       <bottom style="thin">
         <color rgb="FF999999"/>
       </bottom>
-      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
     </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="40">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+  <cellXfs count="51">
+    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFill="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="10" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFill="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="3" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="3" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="2" fillId="3" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment horizontal="left" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="3" fillId="2" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0" shrinkToFit="0" vertical="center" wrapText="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="5" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="4" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="7" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="9" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="9" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="10" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="10" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="11" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="12" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="13" fillId="0" fontId="8" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="14" fillId="4" fontId="9" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="14" fillId="4" fontId="9" numFmtId="10" xfId="0" applyBorder="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="14" fillId="5" fontId="10" numFmtId="0" xfId="0" applyBorder="1" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="10" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="10" fontId="6" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="9" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="10" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+    <xf borderId="0" fillId="0" fontId="11" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="14" fillId="5" fontId="12" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="12" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="9" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf borderId="1" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf borderId="0" fillId="0" fontId="13" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" pivotButton="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle xfId="0" name="Normal" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
-  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
-      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
-    </ext>
-  </extLst>
+  <dxfs count="6">
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF356854"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFF6F8F9"/>
+          <bgColor rgb="FFF6F8F9"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+    <dxf>
+      <border>
+        <left style="thin">
+          <color rgb="FF356854"/>
+        </left>
+        <right style="thin">
+          <color rgb="FF356854"/>
+        </right>
+        <top style="thin">
+          <color rgb="FF356854"/>
+        </top>
+        <bottom style="thin">
+          <color rgb="FF356854"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FFFFFFFF"/>
+        </patternFill>
+      </fill>
+      <border/>
+    </dxf>
+  </dxfs>
+  <tableStyles count="2">
+    <tableStyle count="4" pivot="0" name="liste des taches-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="2" pivot="0" name="detail_avancement-style">
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+    </tableStyle>
+  </tableStyles>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -500,361 +768,248 @@
 </file>
 
 <file path=xl/pivotCache/pivotCacheDefinition1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" r:id="rId1" refreshOnLoad="1" refreshedBy="Harena" refreshedDate="46111.366460532408" refreshedVersion="8" recordCount="19" xr:uid="{00000000-000A-0000-FFFF-FFFF00000000}">
+<pivotCacheDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" invalid="1" refreshOnLoad="1">
   <cacheSource type="worksheet">
-    <worksheetSource ref="B1:K20" sheet="liste des taches"/>
+    <worksheetSource ref="B1:K14" sheet="liste des taches"/>
   </cacheSource>
-  <cacheFields count="10">
+  <cacheFields>
     <cacheField name="Catégorie" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+      <sharedItems>
+        <s v="Infrastructure"/>
+        <s v="Base de données"/>
+        <s v="Backoffice"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Module" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+      <sharedItems>
+        <s v="Setup"/>
+        <s v="Docker"/>
+        <s v="Modélisation"/>
+        <s v="Utilisateurs"/>
+        <s v="Sécurité"/>
+        <s v="Gestion Catégorie"/>
+        <s v="Gestion Article"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Page" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+      <sharedItems>
+        <s v="-"/>
+        <s v="register.php"/>
+        <s v="login.php"/>
+        <s v="logout.php"/>
+        <s v="categorie.php"/>
+        <s v="categorie-add.php"/>
+        <s v="traitement-categorie.php"/>
+        <s v="categorie-edit.php"/>
+        <s v="article-add.php"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Description tâche" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+      <sharedItems>
+        <s v="Init dépôt Git + structure dossiers PHP"/>
+        <s v="Dockerfile (PHP + Apache) + docker-compose"/>
+        <s v="Schéma DB : tables articles, catégories, images"/>
+        <s v="Script SQL de création + données de test"/>
+        <s v="Formulaire d'inscription + hashage mot de passe"/>
+        <s v="Page de connexion + vérification session"/>
+        <s v="Destruction de la session"/>
+        <s v="Sécurisation de toutes les pages BO (check session)"/>
+        <s v="Liste des catégories"/>
+        <s v="Ajout catégorie : formulaire HTML"/>
+        <s v="Traitement ajout catégorie en base"/>
+        <s v="Modification/suppression catégorie"/>
+        <s v="Formulaire ajout article : champs HTML + images + articles référencés"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Type" numFmtId="0">
-      <sharedItems containsBlank="1"/>
+      <sharedItems>
+        <s v="Technique"/>
+        <s v="Base"/>
+        <s v="Métier"/>
+        <s v="Sécurité"/>
+        <s v="Affichage"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Qui" numFmtId="0">
-      <sharedItems containsBlank="1" count="4">
-        <s v="ETU003260"/>
-        <s v="ETU00WWWW"/>
-        <s v="ETU00YYYY"/>
-        <m/>
+      <sharedItems>
+        <s v="ETU003310"/>
+        <s v="ETU003268"/>
       </sharedItems>
     </cacheField>
     <cacheField name="Estimation" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="5" maxValue="50"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
+        <n v="5.0"/>
+        <n v="15.0"/>
+        <n v="10.0"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Temps passé" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="90"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
+        <n v="0.0"/>
+      </sharedItems>
     </cacheField>
     <cacheField name="Reste à faire" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" containsInteger="1" minValue="0" maxValue="40"/>
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
+        <n v="5.0"/>
+        <n v="15.0"/>
+        <n v="10.0"/>
+      </sharedItems>
     </cacheField>
-    <cacheField name="Avancement" numFmtId="0">
-      <sharedItems containsString="0" containsBlank="1" containsNumber="1" minValue="0" maxValue="1"/>
+    <cacheField name="Avancement" numFmtId="10">
+      <sharedItems containsSemiMixedTypes="0" containsString="0" containsNumber="1" containsInteger="1">
+        <n v="0.0"/>
+      </sharedItems>
     </cacheField>
   </cacheFields>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{725AE2AE-9491-48be-B2B4-4EB974FC3084}">
-      <x14:pivotCacheDefinition/>
-    </ext>
-  </extLst>
 </pivotCacheDefinition>
 </file>
 
-<file path=xl/pivotCache/pivotCacheRecords1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotCacheRecords xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" count="19">
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion article"/>
-    <s v="Article-add"/>
-    <s v="Ajout article : code html + images + articles references"/>
-    <s v="Affichage"/>
-    <x v="0"/>
-    <n v="10"/>
-    <n v="10"/>
-    <n v="0"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion article"/>
-    <s v="Traitement-add"/>
-    <s v="Conversion en html avec tinymce"/>
-    <s v="Metier"/>
-    <x v="0"/>
-    <n v="20"/>
-    <n v="0"/>
-    <n v="20"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion article"/>
-    <s v="Traitement-add"/>
-    <s v="Upload images"/>
-    <s v="Metier"/>
-    <x v="0"/>
-    <n v="30"/>
-    <n v="10"/>
-    <n v="20"/>
-    <n v="0.33333333333333331"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion article"/>
-    <s v="Traitement-add"/>
-    <s v="Ajout article : code html en base +articles references en base"/>
-    <s v="Metier"/>
-    <x v="0"/>
-    <n v="10"/>
-    <n v="0"/>
-    <n v="10"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion article"/>
-    <s v="Article-add"/>
-    <s v="Appelle de fonctions du DAO"/>
-    <s v="Integration"/>
-    <x v="0"/>
-    <n v="50"/>
-    <n v="10"/>
-    <n v="40"/>
-    <n v="0.2"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie"/>
-    <s v="Liste"/>
-    <s v="Integration"/>
-    <x v="1"/>
-    <n v="25"/>
-    <n v="0"/>
-    <n v="25"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie-add"/>
-    <s v="Ajout"/>
-    <s v="Affichage"/>
-    <x v="2"/>
-    <n v="10"/>
-    <n v="90"/>
-    <n v="0"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie-add"/>
-    <s v="Ajout"/>
-    <s v="Metier"/>
-    <x v="1"/>
-    <n v="5"/>
-    <n v="30"/>
-    <n v="0"/>
-    <n v="1"/>
-  </r>
-  <r>
-    <s v="Backoffice"/>
-    <s v="Gestion Categorie"/>
-    <s v="Categorie-add"/>
-    <s v="Ajout"/>
-    <s v="Base"/>
-    <x v="1"/>
-    <n v="5"/>
-    <n v="0"/>
-    <n v="5"/>
-    <n v="0"/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-  <r>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-    <x v="3"/>
-    <m/>
-    <m/>
-    <m/>
-    <m/>
-  </r>
-</pivotCacheRecords>
-</file>
-
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{00000000-0007-0000-0200-000000000000}" name="Recap" cacheId="4" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0" dataCaption="" updatedVersion="8" compact="0" compactData="0">
-  <location ref="A1:D7" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
-  <pivotFields count="10">
-    <pivotField name="Catégorie" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="Module" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="Page" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="Description tâche" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="Type" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="Qui" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
-      <items count="5">
-        <item n="ETU003268" x="0"/>
-        <item n="ETU003310" x="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" name="Recap" cacheId="0" dataCaption="" compact="0" compactData="0">
+  <location ref="A1:D4" firstHeaderRow="0" firstDataRow="2" firstDataCol="0"/>
+  <pivotFields>
+    <pivotField name="Catégorie" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item x="1"/>
         <item x="2"/>
-        <item x="3"/>
         <item t="default"/>
       </items>
     </pivotField>
-    <pivotField name="Estimation" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="Temps passé" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="Reste à faire" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
-    <pivotField name="Avancement" compact="0" numFmtId="10" outline="0" multipleItemSelectionAllowed="1" showAll="0"/>
+    <pivotField name="Module" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Page" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Description tâche" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Type" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Qui" axis="axisRow" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0" sortType="ascending">
+      <items>
+        <item x="1"/>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Estimation" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Temps passé" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Reste à faire" dataField="1" compact="0" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField name="Avancement" compact="0" numFmtId="10" outline="0" multipleItemSelectionAllowed="1" showAll="0">
+      <items>
+        <item x="0"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
   </pivotFields>
-  <rowFields count="1">
+  <rowFields>
     <field x="5"/>
   </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colFields count="1">
+  <colFields>
     <field x="-2"/>
   </colFields>
-  <colItems count="3">
-    <i>
-      <x/>
-    </i>
-    <i i="1">
-      <x v="1"/>
-    </i>
-    <i i="2">
-      <x v="2"/>
-    </i>
-  </colItems>
-  <dataFields count="3">
+  <dataFields>
     <dataField name="SUM of Estimation" fld="6" baseField="0"/>
     <dataField name="SUM of Temps passé" fld="7" baseField="0"/>
     <dataField name="SUM of Reste à faire" fld="8" baseField="0"/>
   </dataFields>
-  <pivotTableStyleInfo showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
 </pivotTableDefinition>
 </file>
 
+<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:K28" displayName="Tableau1" name="Tableau1" id="1">
+  <tableColumns count="11">
+    <tableColumn name="Ligne" id="1"/>
+    <tableColumn name="Catégorie" id="2"/>
+    <tableColumn name="Module" id="3"/>
+    <tableColumn name="Page" id="4"/>
+    <tableColumn name="Description tâche" id="5"/>
+    <tableColumn name="Type" id="6"/>
+    <tableColumn name="Qui" id="7"/>
+    <tableColumn name="Estimation" id="8"/>
+    <tableColumn name="Temps passé" id="9"/>
+    <tableColumn name="Reste à faire" id="10"/>
+    <tableColumn name="Avancement" id="11"/>
+  </tableColumns>
+  <tableStyleInfo name="liste des taches-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" headerRowCount="0" ref="A2:A28" displayName="Table_1" name="Table_1" id="2">
+  <tableColumns count="1">
+    <tableColumn name="Column1" id="1"/>
+  </tableColumns>
+  <tableStyleInfo name="detail_avancement-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -1044,58 +1199,56 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
-  <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B1000"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="6" width="12.6328125" customWidth="1"/>
+    <col customWidth="1" min="1" max="6" width="12.63"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15.75" customHeight="1">
+    <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="1" t="s">
-        <v>43</v>
+        <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>44</v>
+        <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15.75" customHeight="1">
+    <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
-        <v>45</v>
+        <v>2</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>46</v>
+        <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15.75" customHeight="1">
+    <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1"/>
       <c r="B3" s="1"/>
     </row>
-    <row r="4" spans="1:2" ht="15.75" customHeight="1">
+    <row r="4" ht="15.75" customHeight="1">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
     </row>
-    <row r="5" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="6" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="7" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="8" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="9" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="10" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="11" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="12" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="13" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="14" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="15" spans="1:2" ht="15.75" customHeight="1"/>
-    <row r="16" spans="1:2" ht="15.75" customHeight="1"/>
+    <row r="5" ht="15.75" customHeight="1"/>
+    <row r="6" ht="15.75" customHeight="1"/>
+    <row r="7" ht="15.75" customHeight="1"/>
+    <row r="8" ht="15.75" customHeight="1"/>
+    <row r="9" ht="15.75" customHeight="1"/>
+    <row r="10" ht="15.75" customHeight="1"/>
+    <row r="11" ht="15.75" customHeight="1"/>
+    <row r="12" ht="15.75" customHeight="1"/>
+    <row r="13" ht="15.75" customHeight="1"/>
+    <row r="14" ht="15.75" customHeight="1"/>
+    <row r="15" ht="15.75" customHeight="1"/>
+    <row r="16" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -2081,539 +2234,1099 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1000"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="5.90625" customWidth="1"/>
-    <col min="2" max="2" width="19" customWidth="1"/>
-    <col min="3" max="3" width="18" customWidth="1"/>
-    <col min="4" max="4" width="12.6328125" customWidth="1"/>
-    <col min="5" max="5" width="59.08984375" customWidth="1"/>
-    <col min="6" max="6" width="12.6328125" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="13.63"/>
+    <col customWidth="1" min="2" max="2" width="19.0"/>
+    <col customWidth="1" min="3" max="3" width="18.0"/>
+    <col customWidth="1" min="4" max="4" width="20.25"/>
+    <col customWidth="1" min="5" max="5" width="59.13"/>
+    <col customWidth="1" min="6" max="6" width="13.5"/>
+    <col customWidth="1" min="7" max="7" width="14.75"/>
+    <col customWidth="1" min="8" max="8" width="18.13"/>
+    <col customWidth="1" min="9" max="9" width="20.25"/>
+    <col customWidth="1" min="10" max="11" width="19.63"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" ht="15.75" customHeight="1">
+    <row r="1" ht="15.75" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="3" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>6</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="J1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K1" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="5">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G2" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="4" t="s">
+      <c r="H2" s="9">
+        <v>5.0</v>
+      </c>
+      <c r="I2" s="10">
+        <f>detail_avancement!B11</f>
+        <v>0</v>
+      </c>
+      <c r="J2" s="10">
+        <f t="shared" ref="J2:J28" si="1">H2-I2</f>
         <v>5</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="4" t="s">
+      <c r="K2" s="11">
+        <f t="shared" ref="K2:K28" si="2">(I2/(I2+J2))</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="D3" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E3" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H3" s="12">
+        <v>15.0</v>
+      </c>
+      <c r="I3" s="10">
+        <f>detail_avancement!B12</f>
+        <v>0</v>
+      </c>
+      <c r="J3" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K3" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="5">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C4" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D4" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G4" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H4" s="12">
+        <v>10.0</v>
+      </c>
+      <c r="I4" s="10">
+        <f>detail_avancement!B13</f>
+        <v>0</v>
+      </c>
+      <c r="J4" s="10">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
+      <c r="K4" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
     </row>
-    <row r="2" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A2" s="5">
-        <v>1</v>
-      </c>
-      <c r="B2" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C2" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D2" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="F2" s="6" t="s">
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="5">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C5" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="G5" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H5" s="9">
+        <v>10.0</v>
+      </c>
+      <c r="I5" s="10">
+        <f>detail_avancement!B14</f>
+        <v>0</v>
+      </c>
+      <c r="J5" s="10">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K5" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="5">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>29</v>
+      </c>
+      <c r="E6" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="H6" s="16">
+        <v>15.0</v>
+      </c>
+      <c r="I6" s="10">
+        <f>detail_avancement!B15</f>
+        <v>0</v>
+      </c>
+      <c r="J6" s="10">
+        <f t="shared" si="1"/>
         <v>15</v>
       </c>
-      <c r="G2" s="39" t="s">
+      <c r="K6" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="5">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="G7" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="H7" s="17">
+        <v>15.0</v>
+      </c>
+      <c r="I7" s="10">
+        <f>detail_avancement!B16</f>
+        <v>0</v>
+      </c>
+      <c r="J7" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K7" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="5">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="14" t="s">
+        <v>35</v>
+      </c>
+      <c r="E8" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="H8" s="17">
+        <v>5.0</v>
+      </c>
+      <c r="I8" s="10">
+        <f>detail_avancement!B17</f>
+        <v>0</v>
+      </c>
+      <c r="J8" s="10">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K8" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="5">
+        <v>8.0</v>
+      </c>
+      <c r="B9" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="14" t="s">
+        <v>17</v>
+      </c>
+      <c r="E9" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="G9" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="H9" s="17">
+        <v>10.0</v>
+      </c>
+      <c r="I9" s="10">
+        <f>detail_avancement!B18</f>
+        <v>0</v>
+      </c>
+      <c r="J9" s="10">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K9" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="5">
+        <v>9.0</v>
+      </c>
+      <c r="B10" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H10" s="12">
+        <v>10.0</v>
+      </c>
+      <c r="I10" s="10">
+        <f>detail_avancement!B19</f>
+        <v>0</v>
+      </c>
+      <c r="J10" s="10">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K10" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="5">
+        <v>10.0</v>
+      </c>
+      <c r="B11" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D11" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="E11" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="H2" s="5">
+      <c r="F11" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H11" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="I11" s="10">
+        <f>detail_avancement!B20</f>
+        <v>0</v>
+      </c>
+      <c r="J11" s="10">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K11" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="5">
+        <v>11.0</v>
+      </c>
+      <c r="B12" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H12" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="I12" s="10">
+        <f>detail_avancement!B21</f>
+        <v>0</v>
+      </c>
+      <c r="J12" s="10">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K12" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="5">
+        <v>12.0</v>
+      </c>
+      <c r="B13" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>47</v>
+      </c>
+      <c r="F13" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H13" s="12">
+        <v>10.0</v>
+      </c>
+      <c r="I13" s="10">
+        <f>detail_avancement!B22</f>
+        <v>0</v>
+      </c>
+      <c r="J13" s="10">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="I2" s="7">
+      <c r="K13" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="5">
+        <v>13.0</v>
+      </c>
+      <c r="B14" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D14" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E14" s="7" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G14" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H14" s="12">
+        <v>10.0</v>
+      </c>
+      <c r="I14" s="10">
+        <f>detail_avancement!B23</f>
+        <v>0</v>
+      </c>
+      <c r="J14" s="10">
+        <f t="shared" si="1"/>
         <v>10</v>
       </c>
-      <c r="J2" s="7">
-        <f t="shared" ref="J2:J7" si="0">H2-I2</f>
-        <v>0</v>
-      </c>
-      <c r="K2" s="8">
+      <c r="K14" s="11">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A3" s="5">
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="5">
+        <v>14.0</v>
+      </c>
+      <c r="B15" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D15" s="7" t="s">
+        <v>49</v>
+      </c>
+      <c r="E15" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H15" s="12">
+        <v>20.0</v>
+      </c>
+      <c r="I15" s="10">
+        <f>detail_avancement!B24</f>
+        <v>0</v>
+      </c>
+      <c r="J15" s="10">
+        <f t="shared" si="1"/>
+        <v>20</v>
+      </c>
+      <c r="K15" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="5">
+        <v>15.0</v>
+      </c>
+      <c r="B16" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C16" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>53</v>
+      </c>
+      <c r="F16" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G16" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H16" s="12">
+        <v>15.0</v>
+      </c>
+      <c r="I16" s="10">
+        <f>detail_avancement!B25</f>
+        <v>0</v>
+      </c>
+      <c r="J16" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K16" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="5">
+        <v>16.0</v>
+      </c>
+      <c r="B17" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C17" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D17" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="E17" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="F17" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G17" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H17" s="12">
+        <v>10.0</v>
+      </c>
+      <c r="I17" s="10">
+        <f>detail_avancement!B26</f>
+        <v>0</v>
+      </c>
+      <c r="J17" s="10">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K17" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="5">
+        <v>17.0</v>
+      </c>
+      <c r="B18" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C18" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D18" s="7" t="s">
+        <v>55</v>
+      </c>
+      <c r="E18" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="F18" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G18" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H18" s="12">
+        <v>10.0</v>
+      </c>
+      <c r="I18" s="10">
+        <f>detail_avancement!B27</f>
+        <v>0</v>
+      </c>
+      <c r="J18" s="10">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K18" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="5">
+        <v>18.0</v>
+      </c>
+      <c r="B19" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="F19" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="G19" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H19" s="12">
+        <v>15.0</v>
+      </c>
+      <c r="I19" s="10">
+        <f>detail_avancement!B28</f>
+        <v>0</v>
+      </c>
+      <c r="J19" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K19" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="5">
+        <v>19.0</v>
+      </c>
+      <c r="B20" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>61</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>62</v>
+      </c>
+      <c r="F20" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G20" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C3" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D3" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E3" s="5" t="s">
+      <c r="H20" s="12">
+        <v>15.0</v>
+      </c>
+      <c r="I20" s="10" t="str">
+        <f>detail_avancement!B29</f>
+        <v/>
+      </c>
+      <c r="J20" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K20" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="5">
+        <v>20.0</v>
+      </c>
+      <c r="B21" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>63</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>65</v>
+      </c>
+      <c r="F21" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G21" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H21" s="12">
+        <v>15.0</v>
+      </c>
+      <c r="I21" s="10" t="str">
+        <f>detail_avancement!B30</f>
+        <v/>
+      </c>
+      <c r="J21" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K21" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="5">
+        <v>21.0</v>
+      </c>
+      <c r="B22" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C22" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D22" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="E22" s="7" t="s">
+        <v>68</v>
+      </c>
+      <c r="F22" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="G22" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H22" s="12">
+        <v>15.0</v>
+      </c>
+      <c r="I22" s="10" t="str">
+        <f>detail_avancement!B31</f>
+        <v/>
+      </c>
+      <c r="J22" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K22" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="5">
+        <v>22.0</v>
+      </c>
+      <c r="B23" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D23" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="E23" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="F23" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G23" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H23" s="12">
+        <v>15.0</v>
+      </c>
+      <c r="I23" s="10" t="str">
+        <f>detail_avancement!B32</f>
+        <v/>
+      </c>
+      <c r="J23" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K23" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="5">
+        <v>23.0</v>
+      </c>
+      <c r="B24" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C24" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E24" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="F24" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G24" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H24" s="12">
+        <v>10.0</v>
+      </c>
+      <c r="I24" s="10" t="str">
+        <f>detail_avancement!B33</f>
+        <v/>
+      </c>
+      <c r="J24" s="10">
+        <f t="shared" si="1"/>
+        <v>10</v>
+      </c>
+      <c r="K24" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="5">
+        <v>24.0</v>
+      </c>
+      <c r="B25" s="6" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D25" s="7" t="s">
+        <v>72</v>
+      </c>
+      <c r="E25" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F25" s="6" t="s">
+        <v>19</v>
+      </c>
+      <c r="G25" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H25" s="12">
+        <v>5.0</v>
+      </c>
+      <c r="I25" s="10" t="str">
+        <f>detail_avancement!B34</f>
+        <v/>
+      </c>
+      <c r="J25" s="10">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K25" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="5">
+        <v>25.0</v>
+      </c>
+      <c r="B26" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C26" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="D26" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="F3" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="39" t="s">
-        <v>43</v>
-      </c>
-      <c r="H3" s="5">
+      <c r="E26" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="F26" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G26" s="6" t="s">
+        <v>2</v>
+      </c>
+      <c r="H26" s="12">
+        <v>15.0</v>
+      </c>
+      <c r="I26" s="10" t="str">
+        <f>detail_avancement!B35</f>
+        <v/>
+      </c>
+      <c r="J26" s="10">
+        <f t="shared" si="1"/>
+        <v>15</v>
+      </c>
+      <c r="K26" s="11">
+        <f t="shared" si="2"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="5">
+        <v>26.0</v>
+      </c>
+      <c r="B27" s="6" t="s">
+        <v>75</v>
+      </c>
+      <c r="C27" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="D27" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E27" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F27" s="6" t="s">
+        <v>78</v>
+      </c>
+      <c r="G27" s="6" t="s">
+        <v>0</v>
+      </c>
+      <c r="H27" s="12">
+        <v>20.0</v>
+      </c>
+      <c r="I27" s="10" t="str">
+        <f>detail_avancement!B36</f>
+        <v/>
+      </c>
+      <c r="J27" s="10">
+        <f t="shared" si="1"/>
         <v>20</v>
       </c>
-      <c r="I3" s="7">
-        <f>detail_avancement!B3</f>
-        <v>0</v>
-      </c>
-      <c r="J3" s="7">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="K3" s="8">
-        <f t="shared" ref="K2:K10" si="1">(I3/(I3+J3))</f>
+      <c r="K27" s="11">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A4" s="5">
-        <v>3</v>
-      </c>
-      <c r="B4" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C4" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D4" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="F4" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="39" t="s">
-        <v>43</v>
-      </c>
-      <c r="H4" s="5">
-        <v>30</v>
-      </c>
-      <c r="I4" s="7">
-        <f>detail_avancement!B4</f>
-        <v>10</v>
-      </c>
-      <c r="J4" s="7">
-        <f t="shared" si="0"/>
-        <v>20</v>
-      </c>
-      <c r="K4" s="8">
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="5">
+        <v>27.0</v>
+      </c>
+      <c r="B28" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="C28" s="19" t="s">
+        <v>82</v>
+      </c>
+      <c r="D28" s="19" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" s="19" t="s">
+        <v>83</v>
+      </c>
+      <c r="F28" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="G28" s="20" t="s">
+        <v>2</v>
+      </c>
+      <c r="H28" s="21">
+        <v>5.0</v>
+      </c>
+      <c r="I28" s="10" t="str">
+        <f>detail_avancement!B37</f>
+        <v/>
+      </c>
+      <c r="J28" s="10">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="K28" s="11">
+        <f t="shared" si="2"/>
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A5" s="5">
-        <v>4</v>
-      </c>
-      <c r="B5" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>16</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>20</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="39" t="s">
-        <v>43</v>
-      </c>
-      <c r="H5" s="5">
-        <v>10</v>
-      </c>
-      <c r="I5" s="7">
-        <f>detail_avancement!B5</f>
-        <v>0</v>
-      </c>
-      <c r="J5" s="7">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="K5" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A6" s="5">
-        <v>5</v>
-      </c>
-      <c r="B6" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C6" s="5" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="G6" s="39" t="s">
-        <v>43</v>
-      </c>
-      <c r="H6" s="5">
-        <v>50</v>
-      </c>
-      <c r="I6" s="7">
-        <f>detail_avancement!B6</f>
-        <v>10</v>
-      </c>
-      <c r="J6" s="7">
-        <f t="shared" si="0"/>
-        <v>40</v>
-      </c>
-      <c r="K6" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A7" s="5">
-        <v>6</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="F7" s="6" t="s">
-        <v>22</v>
-      </c>
-      <c r="G7" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="H7" s="5">
-        <v>25</v>
-      </c>
-      <c r="I7" s="7">
-        <f>detail_avancement!B7</f>
-        <v>0</v>
-      </c>
-      <c r="J7" s="7">
-        <f t="shared" si="0"/>
-        <v>25</v>
-      </c>
-      <c r="K7" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A8" s="5">
-        <v>7</v>
-      </c>
-      <c r="B8" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C8" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="H8" s="5">
-        <v>10</v>
-      </c>
-      <c r="I8" s="7">
-        <f>detail_avancement!B8</f>
-        <v>90</v>
-      </c>
-      <c r="J8" s="7">
-        <v>0</v>
-      </c>
-      <c r="K8" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A9" s="5">
-        <v>8</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C9" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F9" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="G9" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="5">
-        <v>5</v>
-      </c>
-      <c r="I9" s="7">
-        <f>detail_avancement!B9</f>
-        <v>30</v>
-      </c>
-      <c r="J9" s="7">
-        <v>0</v>
-      </c>
-      <c r="K9" s="8">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A10" s="5">
-        <v>9</v>
-      </c>
-      <c r="B10" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="C10" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="5" t="s">
-        <v>26</v>
-      </c>
-      <c r="E10" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>29</v>
-      </c>
-      <c r="G10" s="39" t="s">
-        <v>45</v>
-      </c>
-      <c r="H10" s="5">
-        <v>5</v>
-      </c>
-      <c r="I10" s="7">
-        <f>detail_avancement!B10</f>
-        <v>0</v>
-      </c>
-      <c r="J10" s="7">
-        <f>H10-I10</f>
-        <v>5</v>
-      </c>
-      <c r="K10" s="8">
-        <f t="shared" si="1"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A11" s="9"/>
-      <c r="B11" s="9"/>
-      <c r="C11" s="9"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="9"/>
-      <c r="F11" s="9"/>
-      <c r="G11" s="9"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="9"/>
-      <c r="J11" s="9"/>
-      <c r="K11" s="9"/>
-    </row>
-    <row r="12" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A12" s="9"/>
-      <c r="B12" s="9"/>
-      <c r="C12" s="9"/>
-      <c r="D12" s="9"/>
-      <c r="E12" s="9"/>
-      <c r="F12" s="9"/>
-      <c r="G12" s="9"/>
-      <c r="H12" s="9"/>
-      <c r="I12" s="9"/>
-      <c r="J12" s="9"/>
-      <c r="K12" s="9"/>
-    </row>
-    <row r="13" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A13" s="9"/>
-      <c r="B13" s="9"/>
-      <c r="C13" s="9"/>
-      <c r="D13" s="9"/>
-      <c r="E13" s="9"/>
-      <c r="F13" s="9"/>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9"/>
-      <c r="I13" s="9"/>
-      <c r="J13" s="9"/>
-      <c r="K13" s="9"/>
-    </row>
-    <row r="14" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A14" s="9"/>
-      <c r="B14" s="9"/>
-      <c r="C14" s="9"/>
-      <c r="D14" s="9"/>
-      <c r="E14" s="9"/>
-      <c r="F14" s="9"/>
-      <c r="G14" s="9"/>
-      <c r="H14" s="9"/>
-      <c r="I14" s="9"/>
-      <c r="J14" s="9"/>
-      <c r="K14" s="9"/>
-    </row>
-    <row r="15" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A15" s="9"/>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-      <c r="I15" s="9"/>
-      <c r="J15" s="9"/>
-      <c r="K15" s="9"/>
-    </row>
-    <row r="16" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A16" s="9"/>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9"/>
-      <c r="D16" s="9"/>
-      <c r="E16" s="9"/>
-      <c r="F16" s="9"/>
-      <c r="G16" s="9"/>
-      <c r="H16" s="9"/>
-      <c r="I16" s="9"/>
-      <c r="J16" s="9"/>
-      <c r="K16" s="9"/>
-    </row>
-    <row r="17" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A17" s="9"/>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9"/>
-      <c r="D17" s="9"/>
-      <c r="E17" s="9"/>
-      <c r="F17" s="9"/>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9"/>
-      <c r="I17" s="9"/>
-      <c r="J17" s="9"/>
-      <c r="K17" s="9"/>
-    </row>
-    <row r="18" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A18" s="9"/>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9"/>
-      <c r="D18" s="9"/>
-      <c r="E18" s="9"/>
-      <c r="F18" s="9"/>
-      <c r="G18" s="9"/>
-      <c r="H18" s="9"/>
-      <c r="I18" s="9"/>
-      <c r="J18" s="9"/>
-      <c r="K18" s="9"/>
-    </row>
-    <row r="19" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A19" s="9"/>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
-      <c r="I19" s="9"/>
-      <c r="J19" s="9"/>
-      <c r="K19" s="9"/>
-    </row>
-    <row r="20" spans="1:11" ht="15.75" customHeight="1">
-      <c r="A20" s="9"/>
-      <c r="B20" s="9"/>
-      <c r="C20" s="9"/>
-      <c r="D20" s="9"/>
-      <c r="E20" s="9"/>
-      <c r="F20" s="9"/>
-      <c r="G20" s="9"/>
-      <c r="H20" s="9"/>
-      <c r="I20" s="9"/>
-      <c r="J20" s="9"/>
-      <c r="K20" s="9"/>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="22" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="24" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="26" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="27" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="28" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="29" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="30" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="31" spans="1:11" ht="15.75" customHeight="1"/>
-    <row r="32" spans="1:11" ht="15.75" customHeight="1"/>
+    <row r="29" ht="15.75" customHeight="1"/>
+    <row r="30" ht="15.75" customHeight="1"/>
+    <row r="31" ht="15.75" customHeight="1"/>
+    <row r="32" ht="15.75" customHeight="1"/>
     <row r="33" ht="15.75" customHeight="1"/>
-    <row r="34" ht="15.75" customHeight="1"/>
     <row r="35" ht="15.75" customHeight="1"/>
     <row r="36" ht="15.75" customHeight="1"/>
     <row r="37" ht="15.75" customHeight="1"/>
@@ -2627,7 +3340,23 @@
     <row r="45" ht="15.75" customHeight="1"/>
     <row r="46" ht="15.75" customHeight="1"/>
     <row r="47" ht="15.75" customHeight="1"/>
-    <row r="48" ht="15.75" customHeight="1"/>
+    <row r="48" ht="15.75" customHeight="1">
+      <c r="A48" s="22"/>
+      <c r="B48" s="22"/>
+      <c r="C48" s="22"/>
+      <c r="D48" s="22"/>
+      <c r="E48" s="22"/>
+      <c r="F48" s="22"/>
+      <c r="G48" s="22"/>
+      <c r="H48" s="22"/>
+      <c r="I48" s="22"/>
+      <c r="J48" s="22"/>
+      <c r="K48" s="22"/>
+      <c r="L48" s="22"/>
+      <c r="M48" s="22"/>
+      <c r="N48" s="22"/>
+      <c r="O48" s="22"/>
+    </row>
     <row r="49" ht="15.75" customHeight="1"/>
     <row r="50" ht="15.75" customHeight="1"/>
     <row r="51" ht="15.75" customHeight="1"/>
@@ -3581,124 +4310,92 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <conditionalFormatting sqref="B2:H29">
+    <cfRule type="notContainsBlanks" dxfId="5" priority="1">
+      <formula>LEN(TRIM(B2))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="B6:H9 B26:H29 A29 I29:K29">
+    <cfRule type="notContainsBlanks" dxfId="5" priority="2">
+      <formula>LEN(TRIM(B6))&gt;0</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations>
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="G2:G28">
+      <formula1>"ETU003310,ETU003268"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="B2:B28">
+      <formula1>"Infrastructure,Base de données,Backoffice,Frontoffice,Livraison"</formula1>
+    </dataValidation>
+    <dataValidation type="custom" allowBlank="1" showDropDown="1" sqref="A2:A28 H2:K28">
+      <formula1>AND(ISNUMBER(A2),(NOT(OR(NOT(ISERROR(DATEVALUE(A2))), AND(ISNUMBER(A2), LEFT(CELL("format", A2))="D")))))</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showDropDown="1" showErrorMessage="1" sqref="F2:F28">
+      <formula1>"Technique,Base,Affichage,Métier,Intégration"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1000"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="6" width="12.6328125" customWidth="1"/>
+    <col customWidth="1" min="1" max="3" width="12.63"/>
+    <col customWidth="1" min="4" max="4" width="16.5"/>
+    <col customWidth="1" min="5" max="6" width="12.63"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A1" s="22"/>
-      <c r="B1" s="23" t="s">
-        <v>40</v>
-      </c>
-      <c r="C1" s="24"/>
-      <c r="D1" s="25"/>
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2" ht="15.75" customHeight="1"/>
+    <row r="3" ht="15.75" customHeight="1"/>
+    <row r="4" ht="15.75" customHeight="1"/>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="29"/>
+      <c r="B5" s="29"/>
+      <c r="C5" s="33"/>
+      <c r="D5" s="34"/>
     </row>
-    <row r="2" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A2" s="23" t="s">
-        <v>6</v>
-      </c>
-      <c r="B2" s="22" t="s">
-        <v>30</v>
-      </c>
-      <c r="C2" s="26" t="s">
-        <v>31</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="3" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A3" s="22" t="s">
-        <v>43</v>
-      </c>
-      <c r="B3" s="28">
-        <v>120</v>
-      </c>
-      <c r="C3" s="29">
-        <v>30</v>
-      </c>
-      <c r="D3" s="30">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A4" s="31" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="32">
-        <v>35</v>
-      </c>
-      <c r="C4" s="33">
-        <v>30</v>
-      </c>
-      <c r="D4" s="34">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A5" s="31" t="s">
-        <v>28</v>
-      </c>
-      <c r="B5" s="32">
-        <v>10</v>
-      </c>
-      <c r="C5" s="33">
-        <v>90</v>
-      </c>
-      <c r="D5" s="34">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A6" s="31" t="s">
-        <v>41</v>
-      </c>
-      <c r="B6" s="32"/>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="29"/>
+      <c r="B6" s="29"/>
       <c r="C6" s="33"/>
       <c r="D6" s="34"/>
     </row>
-    <row r="7" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A7" s="35" t="s">
-        <v>42</v>
-      </c>
-      <c r="B7" s="36">
-        <v>165</v>
-      </c>
-      <c r="C7" s="37">
-        <v>150</v>
-      </c>
-      <c r="D7" s="38">
-        <v>120</v>
-      </c>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="35"/>
+      <c r="B7" s="35"/>
+      <c r="C7" s="36"/>
+      <c r="D7" s="37"/>
     </row>
-    <row r="8" spans="1:4" ht="15.75" customHeight="1"/>
-    <row r="9" spans="1:4" ht="15.75" customHeight="1"/>
-    <row r="10" spans="1:4" ht="15.75" customHeight="1"/>
-    <row r="11" spans="1:4" ht="15.75" customHeight="1"/>
-    <row r="12" spans="1:4" ht="15.75" customHeight="1">
-      <c r="A12" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" s="11">
+    <row r="8" ht="15.75" customHeight="1"/>
+    <row r="9" ht="15.75" customHeight="1"/>
+    <row r="10" ht="15.75" customHeight="1"/>
+    <row r="11" ht="15.75" customHeight="1"/>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="38" t="s">
+        <v>14</v>
+      </c>
+      <c r="B12" s="39">
         <f>avancement!D2</f>
-        <v>0.55555555555555558</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" ht="15.75" customHeight="1"/>
-    <row r="14" spans="1:4" ht="15.75" customHeight="1"/>
-    <row r="15" spans="1:4" ht="15.75" customHeight="1"/>
-    <row r="16" spans="1:4" ht="15.75" customHeight="1"/>
+    <row r="13" ht="15.75" customHeight="1"/>
+    <row r="14" ht="15.75" customHeight="1"/>
+    <row r="15" ht="15.75" customHeight="1"/>
+    <row r="16" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -4684,90 +5381,93 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1000"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="15.7265625" customWidth="1"/>
-    <col min="2" max="2" width="17.90625" customWidth="1"/>
-    <col min="3" max="3" width="17" customWidth="1"/>
-    <col min="4" max="4" width="18.26953125" customWidth="1"/>
-    <col min="5" max="5" width="13.7265625" customWidth="1"/>
-    <col min="6" max="6" width="12.6328125" customWidth="1"/>
+    <col customWidth="1" min="1" max="1" width="15.75"/>
+    <col customWidth="1" min="2" max="2" width="17.88"/>
+    <col customWidth="1" min="3" max="3" width="17.0"/>
+    <col customWidth="1" min="4" max="4" width="18.25"/>
+    <col customWidth="1" min="5" max="5" width="13.75"/>
+    <col customWidth="1" min="6" max="6" width="12.63"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A1" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="B1" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="C1" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D1" s="12" t="s">
-        <v>36</v>
-      </c>
-      <c r="E1" s="12" t="s">
-        <v>37</v>
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="40" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" s="40" t="s">
+        <v>89</v>
+      </c>
+      <c r="C1" s="40" t="s">
+        <v>90</v>
+      </c>
+      <c r="D1" s="40" t="s">
+        <v>91</v>
+      </c>
+      <c r="E1" s="40" t="s">
+        <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A2" s="13">
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="41">
         <f>SUM('liste des taches'!H:H)</f>
-        <v>165</v>
-      </c>
-      <c r="B2" s="13">
+        <v>310</v>
+      </c>
+      <c r="B2" s="41">
         <f>SUM('liste des taches'!I:I)</f>
-        <v>150</v>
-      </c>
-      <c r="C2" s="13">
+        <v>0</v>
+      </c>
+      <c r="C2" s="41">
         <f>SUM('liste des taches'!J:J)</f>
-        <v>120</v>
-      </c>
-      <c r="D2" s="14">
+        <v>310</v>
+      </c>
+      <c r="D2" s="42">
         <f>(B2/(B2+C2))</f>
-        <v>0.55555555555555558</v>
-      </c>
-      <c r="E2" s="15">
+        <v>0</v>
+      </c>
+      <c r="E2" s="43">
         <f>((B2+C2)-A2)/A2</f>
-        <v>0.63636363636363635</v>
+        <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A3" s="16"/>
-      <c r="B3" s="16"/>
-      <c r="C3" s="13">
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="44"/>
+      <c r="B3" s="44"/>
+      <c r="C3" s="41">
         <f>C2/60</f>
-        <v>2</v>
-      </c>
-      <c r="D3" s="16" t="s">
-        <v>38</v>
-      </c>
-      <c r="E3" s="16"/>
+        <v>5.166666667</v>
+      </c>
+      <c r="D3" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="E3" s="44"/>
     </row>
-    <row r="4" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="5" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="6" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="7" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="8" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="9" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="10" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="11" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="12" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="13" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="14" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="15" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="16" spans="1:5" ht="15.75" customHeight="1"/>
+    <row r="4" ht="15.75" customHeight="1"/>
+    <row r="5" ht="15.75" customHeight="1"/>
+    <row r="6" ht="15.75" customHeight="1"/>
+    <row r="7" ht="15.75" customHeight="1"/>
+    <row r="8" ht="15.75" customHeight="1"/>
+    <row r="9" ht="15.75" customHeight="1"/>
+    <row r="10" ht="15.75" customHeight="1"/>
+    <row r="11" ht="15.75" customHeight="1"/>
+    <row r="12" ht="15.75" customHeight="1"/>
+    <row r="13" ht="15.75" customHeight="1"/>
+    <row r="14" ht="15.75" customHeight="1"/>
+    <row r="15" ht="15.75" customHeight="1"/>
+    <row r="16" ht="15.75" customHeight="1"/>
     <row r="17" ht="15.75" customHeight="1"/>
     <row r="18" ht="15.75" customHeight="1"/>
     <row r="19" ht="15.75" customHeight="1"/>
@@ -5753,169 +6453,451 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1000"/>
-  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15" customHeight="1"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="6" width="12.6328125" customWidth="1"/>
+    <col customWidth="1" min="1" max="6" width="12.63"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A1" s="17" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="18" t="s">
-        <v>39</v>
-      </c>
-      <c r="C1" s="19">
-        <v>46111</v>
-      </c>
-      <c r="D1" s="19">
-        <v>46112</v>
-      </c>
-      <c r="E1" s="19"/>
+    <row r="1" ht="15.75" customHeight="1">
+      <c r="A1" s="45" t="s">
+        <v>4</v>
+      </c>
+      <c r="B1" s="46" t="s">
+        <v>94</v>
+      </c>
+      <c r="C1" s="47">
+        <v>46111.0</v>
+      </c>
+      <c r="D1" s="47">
+        <v>46112.0</v>
+      </c>
+      <c r="E1" s="47"/>
     </row>
-    <row r="2" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A2" s="20">
-        <v>1</v>
-      </c>
-      <c r="B2" s="13">
-        <f t="shared" ref="B2:B10" si="0">SUM(D2:P2)</f>
-        <v>20</v>
-      </c>
-      <c r="C2" s="16"/>
-      <c r="D2" s="20">
-        <v>20</v>
-      </c>
-      <c r="E2" s="16"/>
+    <row r="2" ht="15.75" customHeight="1">
+      <c r="A2" s="48">
+        <v>1.0</v>
+      </c>
+      <c r="B2" s="41">
+        <f t="shared" ref="B2:B28" si="1">SUM(C2:D2)</f>
+        <v>0</v>
+      </c>
+      <c r="C2" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D2" s="50">
+        <v>0.0</v>
+      </c>
+      <c r="E2" s="44"/>
     </row>
-    <row r="3" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A3" s="20">
-        <v>2</v>
-      </c>
-      <c r="B3" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="C3" s="16"/>
-      <c r="D3" s="16"/>
-      <c r="E3" s="16"/>
+    <row r="3" ht="15.75" customHeight="1">
+      <c r="A3" s="48">
+        <v>2.0</v>
+      </c>
+      <c r="B3" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C3" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D3" s="50">
+        <v>0.0</v>
+      </c>
+      <c r="E3" s="44"/>
     </row>
-    <row r="4" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A4" s="20">
-        <v>3</v>
-      </c>
-      <c r="B4" s="13">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="C4" s="20">
-        <v>20</v>
-      </c>
-      <c r="D4" s="20">
-        <v>10</v>
-      </c>
-      <c r="E4" s="16"/>
+    <row r="4" ht="15.75" customHeight="1">
+      <c r="A4" s="48">
+        <v>3.0</v>
+      </c>
+      <c r="B4" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C4" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D4" s="50">
+        <v>0.0</v>
+      </c>
+      <c r="E4" s="44"/>
     </row>
-    <row r="5" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A5" s="20">
-        <v>4</v>
-      </c>
-      <c r="B5" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="C5" s="16"/>
-      <c r="D5" s="16"/>
-      <c r="E5" s="16"/>
+    <row r="5" ht="15.75" customHeight="1">
+      <c r="A5" s="48">
+        <v>4.0</v>
+      </c>
+      <c r="B5" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C5" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D5" s="50">
+        <v>0.0</v>
+      </c>
+      <c r="E5" s="44"/>
     </row>
-    <row r="6" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A6" s="20">
-        <v>5</v>
-      </c>
-      <c r="B6" s="13">
-        <f t="shared" si="0"/>
-        <v>10</v>
-      </c>
-      <c r="C6" s="16"/>
-      <c r="D6" s="21">
-        <v>10</v>
-      </c>
-      <c r="E6" s="16"/>
+    <row r="6" ht="15.75" customHeight="1">
+      <c r="A6" s="48">
+        <v>5.0</v>
+      </c>
+      <c r="B6" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C6" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D6" s="50">
+        <v>0.0</v>
+      </c>
+      <c r="E6" s="44"/>
     </row>
-    <row r="7" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A7" s="20">
-        <v>6</v>
-      </c>
-      <c r="B7" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="C7" s="16"/>
-      <c r="D7" s="16"/>
-      <c r="E7" s="16"/>
+    <row r="7" ht="15.75" customHeight="1">
+      <c r="A7" s="48">
+        <v>6.0</v>
+      </c>
+      <c r="B7" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C7" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D7" s="50">
+        <v>0.0</v>
+      </c>
+      <c r="E7" s="44"/>
     </row>
-    <row r="8" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A8" s="20">
-        <v>7</v>
-      </c>
-      <c r="B8" s="13">
-        <f t="shared" si="0"/>
-        <v>90</v>
-      </c>
-      <c r="C8" s="16"/>
-      <c r="D8" s="21">
-        <v>90</v>
-      </c>
-      <c r="E8" s="16"/>
+    <row r="8" ht="15.75" customHeight="1">
+      <c r="A8" s="48">
+        <v>7.0</v>
+      </c>
+      <c r="B8" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C8" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D8" s="50">
+        <v>0.0</v>
+      </c>
+      <c r="E8" s="44"/>
     </row>
-    <row r="9" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" s="13">
-        <f t="shared" si="0"/>
-        <v>30</v>
-      </c>
-      <c r="D9" s="1">
-        <v>30</v>
+    <row r="9" ht="15.75" customHeight="1">
+      <c r="A9" s="48">
+        <v>8.0</v>
+      </c>
+      <c r="B9" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C9" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D9" s="50">
+        <v>0.0</v>
       </c>
     </row>
-    <row r="10" spans="1:5" ht="15.75" customHeight="1">
-      <c r="A10" s="1">
-        <v>9</v>
-      </c>
-      <c r="B10" s="13">
-        <f t="shared" si="0"/>
-        <v>0</v>
+    <row r="10" ht="15.75" customHeight="1">
+      <c r="A10" s="48">
+        <v>9.0</v>
+      </c>
+      <c r="B10" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C10" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D10" s="50">
+        <v>0.0</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="12" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="13" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="14" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="15" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="16" spans="1:5" ht="15.75" customHeight="1"/>
-    <row r="17" ht="15.75" customHeight="1"/>
-    <row r="18" ht="15.75" customHeight="1"/>
-    <row r="19" ht="15.75" customHeight="1"/>
-    <row r="20" ht="15.75" customHeight="1"/>
-    <row r="21" ht="15.75" customHeight="1"/>
-    <row r="22" ht="15.75" customHeight="1"/>
-    <row r="23" ht="15.75" customHeight="1"/>
-    <row r="24" ht="15.75" customHeight="1"/>
-    <row r="25" ht="15.75" customHeight="1"/>
-    <row r="26" ht="15.75" customHeight="1"/>
-    <row r="27" ht="15.75" customHeight="1"/>
-    <row r="28" ht="15.75" customHeight="1"/>
+    <row r="11" ht="15.75" customHeight="1">
+      <c r="A11" s="48">
+        <v>10.0</v>
+      </c>
+      <c r="B11" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C11" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D11" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="12" ht="15.75" customHeight="1">
+      <c r="A12" s="48">
+        <v>11.0</v>
+      </c>
+      <c r="B12" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C12" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D12" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="13" ht="15.75" customHeight="1">
+      <c r="A13" s="48">
+        <v>12.0</v>
+      </c>
+      <c r="B13" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C13" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D13" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="14" ht="15.75" customHeight="1">
+      <c r="A14" s="48">
+        <v>13.0</v>
+      </c>
+      <c r="B14" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C14" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D14" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="15" ht="15.75" customHeight="1">
+      <c r="A15" s="48">
+        <v>14.0</v>
+      </c>
+      <c r="B15" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C15" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D15" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="16" ht="15.75" customHeight="1">
+      <c r="A16" s="48">
+        <v>15.0</v>
+      </c>
+      <c r="B16" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C16" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D16" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="17" ht="15.75" customHeight="1">
+      <c r="A17" s="48">
+        <v>16.0</v>
+      </c>
+      <c r="B17" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C17" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D17" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="18" ht="15.75" customHeight="1">
+      <c r="A18" s="48">
+        <v>17.0</v>
+      </c>
+      <c r="B18" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C18" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D18" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="19" ht="15.75" customHeight="1">
+      <c r="A19" s="48">
+        <v>18.0</v>
+      </c>
+      <c r="B19" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C19" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D19" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="20" ht="15.75" customHeight="1">
+      <c r="A20" s="48">
+        <v>19.0</v>
+      </c>
+      <c r="B20" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C20" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D20" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="21" ht="15.75" customHeight="1">
+      <c r="A21" s="48">
+        <v>20.0</v>
+      </c>
+      <c r="B21" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C21" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D21" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="22" ht="15.75" customHeight="1">
+      <c r="A22" s="48">
+        <v>21.0</v>
+      </c>
+      <c r="B22" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C22" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D22" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="23" ht="15.75" customHeight="1">
+      <c r="A23" s="48">
+        <v>22.0</v>
+      </c>
+      <c r="B23" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C23" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D23" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="24" ht="15.75" customHeight="1">
+      <c r="A24" s="48">
+        <v>23.0</v>
+      </c>
+      <c r="B24" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C24" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D24" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="25" ht="15.75" customHeight="1">
+      <c r="A25" s="48">
+        <v>24.0</v>
+      </c>
+      <c r="B25" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C25" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D25" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="26" ht="15.75" customHeight="1">
+      <c r="A26" s="48">
+        <v>25.0</v>
+      </c>
+      <c r="B26" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C26" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D26" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="27" ht="15.75" customHeight="1">
+      <c r="A27" s="48">
+        <v>26.0</v>
+      </c>
+      <c r="B27" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C27" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D27" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
+    <row r="28" ht="15.75" customHeight="1">
+      <c r="A28" s="48">
+        <v>27.0</v>
+      </c>
+      <c r="B28" s="41">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+      <c r="C28" s="49">
+        <v>0.0</v>
+      </c>
+      <c r="D28" s="50">
+        <v>0.0</v>
+      </c>
+    </row>
     <row r="29" ht="15.75" customHeight="1"/>
     <row r="30" ht="15.75" customHeight="1"/>
     <row r="31" ht="15.75" customHeight="1"/>
@@ -6889,6 +7871,12 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup orientation="landscape"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
</xml_diff>